<commit_message>
docs(security): closure complete — final closure report, single-file master hand-over for independent review, updated registers, ISO 27001 v1.1 and SOC 2 v1.1 with control matrices, third independent retest evidence
Records that the GitHub repository is public (deploy and verify before pushing), the four migrations and
their order, the commit/count reconciliation, and that production remains NOT remediated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/security/CKAM_SOC2_CONTROL_MATRIX.xlsx
+++ b/docs/security/CKAM_SOC2_CONTROL_MATRIX.xlsx
@@ -10,7 +10,7 @@
     <sheet name="SOC2 Controls" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SOC2 Controls'!$A$1:$M$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SOC2 Controls'!$A$1:$N$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,7 @@
     <col width="48" customWidth="1" min="11" max="11"/>
     <col width="48" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,6 +515,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Previous Status (2026-10-15)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -553,7 +559,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>NOT EVIDENCED; docs/security/policies/01_Information_Security_Policy.md (DRAFT - MANAGEMENT APPROVAL REQUIRED; not evidence)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -568,15 +574,20 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>No approved policy set</t>
+          <t>Policy set exists only as DRAFT (15 documents, 0 approved, 0 operating)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>EXT-17</t>
+          <t>Approve the drafts (SD-16, EXT-17)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -620,7 +631,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/CKAM_PRODUCTION_SERVER_CHECKLIST.md (owners not yet assigned)</t>
+          <t>docs/ai/CKAM_PRODUCTION_SERVER_CHECKLIST.md (owners not yet assigned); docs/security/policies/01_Information_Security_Policy.md roles (DRAFT)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -635,7 +646,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Roles unassigned</t>
+          <t>Roles drafted, nobody appointed</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -644,6 +655,11 @@
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -715,6 +731,11 @@
           <t>NOT READY</t>
         </is>
       </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -754,7 +775,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>NOT EVIDENCED; docs/security/policies/10_Security_Awareness_Plan.md (DRAFT)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -778,6 +799,11 @@
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -849,6 +875,11 @@
           <t>PARTIAL</t>
         </is>
       </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -916,6 +947,11 @@
           <t>PARTIAL</t>
         </is>
       </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -983,6 +1019,11 @@
           <t>NOT READY</t>
         </is>
       </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1022,7 +1063,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>docs/security/CKAM_ISO27001_READINESS.md (draft register, 31 risks)</t>
+          <t>docs/security/CKAM_ISO27001_READINESS.md (draft register, 31 risks); docs/security/CKAM_ISO27001_READINESS.md section 9 (draft register re-scored 2026-10-16: 40 risks); docs/security/policies/12_Risk_Management_Procedure.md (DRAFT)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1046,6 +1087,11 @@
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1117,6 +1163,11 @@
           <t>PARTIAL</t>
         </is>
       </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1156,7 +1207,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>docs/security/CKAM_SECURITY_BASELINE.md; backend/tests/observability/test_coverage_walker.py</t>
+          <t>docs/security/CKAM_SECURITY_BASELINE.md; backend/tests/observability/test_coverage_walker.py; docs/security/CKAM_SECURITY_BASELINE.md (closure rules added 2026-10-16)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1180,6 +1231,11 @@
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1223,7 +1279,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>NOT EVIDENCED; docs/security/policies/13_Internal_Audit_Checklist.md (DRAFT, never used)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1247,6 +1303,11 @@
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -1290,7 +1351,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/REVIEW_FINDINGS.md; docs/security/evidence/access/findings.csv; docs/security/CKAM_EXTERNAL_SECURITY_ACTIONS.md</t>
+          <t>docs/ai/REVIEW_FINDINGS.md; docs/security/evidence/access/findings.csv; docs/security/CKAM_EXTERNAL_SECURITY_ACTIONS.md; docs/security/CKAM_SECURITY_CLOSURE_REGISTER.md; docs/security/CKAM_SECURITY_FINDINGS_REGISTER.md</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1305,7 +1366,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>No single owned tracker with dates</t>
+          <t>Trackers exist as documents; no owned tracker with due dates operating</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1314,6 +1375,11 @@
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1357,7 +1423,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/DEVELOPMENT_GUARDRAILS.md; docs/security/CKAM_SECURITY_BASELINE.md</t>
+          <t>docs/ai/DEVELOPMENT_GUARDRAILS.md; docs/security/CKAM_SECURITY_BASELINE.md; Baseline updated 2026-10-16 (still not approved)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1381,6 +1447,11 @@
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1452,6 +1523,11 @@
           <t>NOT READY</t>
         </is>
       </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1491,7 +1567,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/access/authz_matrix.csv (217 routes x 11 personas); docs/security/evidence/access/tests.csv (0 privilege escalation)</t>
+          <t>docs/security/evidence/access/authz_matrix.csv (217 routes x 11 personas); docs/security/evidence/access/tests.csv (0 privilege escalation); docs/security/evidence/closure/retest2/access/authz_matrix.csv (final code: 217 routes x 14 identities = 3,038 cells, 0 escalations)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1515,6 +1591,11 @@
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -1558,7 +1639,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/access/tests.csv (208 IDOR/BOLA cases); backend/tests/core/test_security_read_scope.py; AC-1, AC-2, IF-03 FIXED and retested (commits 77431ba, 7e57844)</t>
+          <t>docs/security/evidence/access/tests.csv (208 IDOR/BOLA cases); backend/tests/core/test_security_read_scope.py; AC-1, AC-2, IF-03 FIXED and retested (commits 77431ba, 7e57844); docs/security/evidence/closure/retest2/access/tests.csv (319 cases, 318 PASS, 1 OBS)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1573,7 +1654,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Fixes are local commits; production 3b5e842 does not have them</t>
+          <t>Only deployment is missing: production 3b5e842 lacks the AC-1, AC-2 and IF-03 fixes</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1582,6 +1663,11 @@
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1625,7 +1711,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>audit_log CREATE rows; SECURITY PASSWORD_RESET rows; docs/security/evidence/auth/tests.csv AU-T050</t>
+          <t>audit_log CREATE rows; SECURITY PASSWORD_RESET rows; docs/security/evidence/auth/tests.csv AU-T050; docs/security/policies/03_Joiner_Mover_Leaver_Procedure.md and templates/joiner_mover_leaver_record.md (DRAFT)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1649,6 +1735,11 @@
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1692,7 +1783,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/auth/test_vapt_sessions.py (AU-07 FIXED: token_version ends sessions on deactivation, login switch-off, role/area/company/password change)</t>
+          <t>backend/tests/auth/test_vapt_sessions.py (AU-07 FIXED: token_version ends sessions on deactivation, login switch-off, role/area/company/password change); backend/tests/auth/test_wpa2_token_version_atomic.py (atomic session version; server-side refresh sessions ended too); docs/security/policies/03 (DRAFT)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1716,6 +1807,11 @@
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1759,7 +1855,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>GET /api/asset-users/export (exists); review sign-off NOT EVIDENCED</t>
+          <t>GET /api/asset-users/export (exists); review sign-off NOT EVIDENCED; docs/security/policies/11_Periodic_Access_Review_Procedure.md and templates/access_review_record.md (DRAFT, never run)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1783,6 +1879,11 @@
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -1854,6 +1955,11 @@
           <t>PARTIAL</t>
         </is>
       </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1893,7 +1999,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/auth/tests.csv AU-T044..AU-T049; backend/app/auth/password_policy.py; backend/tests/auth/test_vapt_password_policy.py (AU-08 FIXED)</t>
+          <t>docs/security/evidence/auth/tests.csv AU-T044..AU-T049; backend/app/auth/password_policy.py; backend/tests/auth/test_vapt_password_policy.py (AU-08 FIXED); stricter name look-alike password check and a refusal text naming both secret rules (7b039fb); docs/security/policies/02_Access_Control_Policy.md (DRAFT)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1917,6 +2023,11 @@
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -1988,6 +2099,11 @@
           <t>NOT READY</t>
         </is>
       </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2027,7 +2143,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>backend/app/core/rate_limit.py; backend/tests/auth/test_rate_limit.py, test_vapt_login.py (AU-01, AU-03, AU-16 FIXED; AU-04 MITIGATED; AU-02 ACCEPTED); audit_log LOGIN_FAILED / LOCKED rows</t>
+          <t>backend/app/core/rate_limit.py; backend/tests/auth/test_rate_limit.py, test_vapt_login.py (AU-01, AU-03, AU-16 FIXED; AU-04 MITIGATED; AU-02 ACCEPTED); audit_log LOGIN_FAILED / LOCKED rows; docs/security/evidence/closure/retest2/sessions/raw/a3_ratelimit.json and a7_timing.json (rate limits via nginx and direct, timing medians within 3.8 ms); docs/security/evidence/closure/backend/AU-04_OPTIONS.md</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2042,7 +2158,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Not deployed; residual lock-out DoS (AU-04); users behind one NAT share the per-address limit</t>
+          <t>Not deployed; AU-04 lock-out DoS needs an owner decision (options A/B/C, recommendation C); per-address limit shared behind office NAT needs a per-office policy (EXT-40, EXT-49)</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2051,6 +2167,11 @@
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -2074,7 +2195,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>15-minute access token; 8-hour refresh; logout revokes refresh token</t>
+          <t>15-minute access token; 8-hour refresh; refresh token rotated once with server-side reuse detection (auth_session stores only a SHA-256 of the token id; reuse =&gt; 401, every session of that person ended, REFRESH_REUSE row; 10 s grace for parallel tabs, REFRESH_DUPLICATE row); logout signs out everywhere; token_version raised atomically</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2094,7 +2215,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/auth/test_vapt_sessions.py; migration f9a1c3e5b7d2 (token_version); AU-05, AU-07 FIXED; AU-06 MITIGATED (rotation per refresh; an old rotated token stays valid until sign-out or expiry)</t>
+          <t>backend/tests/auth/test_vapt_sessions.py; migration f9a1c3e5b7d2 (token_version); AU-05, AU-07 FIXED; AU-06 MITIGATED (rotation per refresh; an old rotated token stays valid until sign-out or expiry); backend/tests/auth/test_wpa2_refresh_reuse.py; backend/tests/auth/test_wpa2_token_version_atomic.py; migration b5d7f9a1c3e5 (auth_session); docs/security/evidence/closure/retest2/sessions/raw/a1_refresh.json, a2_revocation.json (AU-06 FIXED in code)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2109,7 +2230,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Not deployed; AU-06 residual</t>
+          <t>Not deployed; residual 10 s grace window (R-34); no absolute session lifetime (decision, EXT-50)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2118,6 +2239,11 @@
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -2189,6 +2315,11 @@
           <t>NOT READY</t>
         </is>
       </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2256,6 +2387,11 @@
           <t>NOT READY</t>
         </is>
       </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2295,7 +2431,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (shared\.env and nas.pw Administrators/SYSTEM only); IF-01 exposure</t>
+          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (shared\.env and nas.pw Administrators/SYSTEM only); IF-01 exposure; docs/security/CKAM_URGENT_PRODUCTION_SECURITY_RUNBOOK.md phases 8-11 (rotation prepared, NOT executed)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2319,6 +2455,11 @@
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -2362,7 +2503,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md</t>
+          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md; docs/security/CKAM_HTTPS_IMPLEMENTATION_PLAN.md (prepared)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2386,6 +2527,11 @@
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -2457,6 +2603,11 @@
           <t>NOT READY</t>
         </is>
       </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2496,7 +2647,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/input/raw_sql_review.md section 8; backend/tests/test_static_frontend.py; backend/tests/documents/test_vapt_content_check.py; IF-01, IN-02, IN-03 FIXED and retested</t>
+          <t>docs/security/evidence/input/raw_sql_review.md section 8; backend/tests/test_static_frontend.py; backend/tests/documents/test_vapt_content_check.py; IF-01, IN-02, IN-03 FIXED and retested; backend/tests/test_static_frontend_windows.py (lexical Windows-path refusal before any filesystem call); backend/tests/test_static_frontend_spa_assets.py; docs/security/evidence/closure/windows/ (native Windows: fixed code refused 28 of 28 payloads, 0 leaks)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2511,7 +2662,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>IF-01 still live in production until deploy and secret rotation</t>
+          <t>Not deployed: production 3b5e842 still serves files outside the frontend folder (IF-01) until EXT-01; secret rotation is CC6-13</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2520,6 +2671,11 @@
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -2543,7 +2699,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Content-Security-Policy and Permissions-Policy headers; no source maps in builds; API docs off in production; request-size limits (64 KB sign-in, 5 MB JSON, 16 MB uploads, 413); unknown ENVIRONMENT_NAME treated as production</t>
+          <t>Content-Security-Policy (self-hosted fonts, no Google hosts) and Permissions-Policy; security headers exactly once; no source maps; API docs off with JSON 404 for docs paths and unknown /api; request-size limits (64 KB sign-in, 5 MB JSON, 16 MB uploads, 413); unset or unknown ENVIRONMENT_NAME treated as production; no server banner; uvicorn without proxy-header trust</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2563,7 +2719,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_vapt_headers_and_docs.py; backend/tests/core/test_body_limit.py; backend/tests/core/test_production_secret_guard.py; frontend/vite.config.ts; frontend/e2e/security.spec.ts (AU-11, AU-12, AU-14, AU-15, IF-14, N1, N4 FIXED)</t>
+          <t>backend/tests/test_vapt_headers_and_docs.py; backend/tests/core/test_body_limit.py; backend/tests/core/test_production_secret_guard.py; frontend/vite.config.ts; frontend/e2e/security.spec.ts (AU-11, AU-12, AU-14, AU-15, IF-14, N1, N4 FIXED); frontend/scripts/check-build-security.mjs (npm run check:build: 0 .map files, no Google host); frontend/scripts/check-nginx-live.mjs; frontend/src/security/nginx-config.test.ts; backend/tests/core/test_n2_forwarded_for.py; docs/security/evidence/closure/wpf/WPF_RESULTS.md</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2578,7 +2734,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Not deployed; uvicorn trusts X-Forwarded-For from 127.0.0.1 (N2) until started with --no-proxy-headers</t>
+          <t>Not deployed; the production launcher must start uvicorn with --no-proxy-headers --no-server-header (EXT-38)</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2587,6 +2743,11 @@
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -2595,141 +2756,151 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CC6-17</t>
+          <t>CC6-19</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Security (CC6 Physical access)</t>
+          <t>Security (CC6 Logical access)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Equipment is disposed of securely</t>
+          <t>The application database account has least privilege</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Wipe before disposal; CKAM Disposed/Scrapped status with certificate</t>
+          <t>Owner / migrator / runtime role split: the runtime role owns nothing, cannot TRUNCATE, ALTER, DROP or disable triggers, has INSERT/SELECT only on append-only tables and USAGE/SELECT only on sequences; role settings RESET ALL; ops/db/check_least_privilege.sql re-run after every deploy</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DBA; Dev lead</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per deploy (check); continuous (grants)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>CKAM; organisation</t>
+          <t>PostgreSQL 10.0.0.205</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>CKAM disposal statuses exist; wiping NOT EVIDENCED</t>
+          <t>ops/db/role_split.sql, role_split_verify.sql, check_least_privilege.sql, ROLE_SPLIT_RUNBOOK.md; docs/security/evidence/closure/db/WPB_RESULTS.md (disposable DB: runtime role 7/7 needed actions, 40/40 forbidden refused; verify 45/45; 34 least-privilege checks); docs/security/evidence/closure/retest2/infra/raw/db6b_03_runtime_attacks.out.txt; backend/tests/security/test_least_privilege_role_split.py</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES (scripts, disposable DB) / NO (production)</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>NO (never run in production; the per-deploy check output would become the evidence)</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Wiping not evidenced</t>
+          <t>Production runtime role ckassetapp still owns the tables; the DBA must run the updated scripts (sequence-privilege fix, RESET ALL)</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Procedure + certificate upload</t>
+          <t>EXT-07, EXT-45, EXT-46</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>NEW 2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CC7-01</t>
+          <t>CC6-17</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Security (CC7 System operations)</t>
+          <t>Security (CC6 Physical access)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Security events are logged</t>
+          <t>Equipment is disposed of securely</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Sign-in, failed sign-in, lockout, logout, password change/reset, access change, permission denied, suspicious input</t>
+          <t>Wipe before disposal; CKAM Disposed/Scrapped status with certificate</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>CKAM; organisation</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md section 2; docs/security/evidence/auth/tests.csv AU-T096</t>
+          <t>CKAM disposal statuses exist; wiping NOT EVIDENCED</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - audit_log kept forever; no observation period</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Wiping not evidenced</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Procedure + certificate upload</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CC7-02</t>
+          <t>CC7-01</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2739,17 +2910,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Audit records cannot be altered</t>
+          <t>Security events are logged</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Append-only UPDATE/DELETE/TRUNCATE guards on audit_log, asset_event, asset_field_change, master_audit; audit purge refused for rows younger than 5 years; owner/runtime role split</t>
+          <t>Sign-in, failed sign-in, lockout, logout, password change/reset, access change, permission denied, suspicious input</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>DBA; Dev lead</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2759,44 +2930,49 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/infra/db_03_append_only_privilege_tests.out.txt; db_04_least_priv_flag_bypass.out.txt; migration a3c5e7f9b1d4; backend/tests/observability/test_vapt_append_only.py (IF-05/IF-06/AU-10 MITIGATED)</t>
+          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md section 2; docs/security/evidence/auth/tests.csv AU-T096; Closure (not deployed): SECURITY rows REFRESH_REUSE, REFRESH_DUPLICATE and RATE_LIMITED added next to LOGIN_FAILED, LOCKED, INVALID_TOKEN, PERMISSION_DENIED</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>N/A (configuration)</t>
+          <t>SOURCE EXISTS - audit_log kept forever; no observation period</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Owner or superuser can still drop triggers; not deployed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>EXT-07 role split; EXT-01</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CC7-03</t>
+          <t>CC7-02</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2806,64 +2982,69 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Audit logs are reviewed</t>
+          <t>Audit records cannot be altered</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Weekly review of SECURITY rows (failed logins, lockouts, access changes, permission denied)</t>
+          <t>Append-only UPDATE/DELETE/TRUNCATE guards on audit_log, asset_event, asset_field_change, master_audit; audit purge refused for rows younger than 5 years; owner/runtime role split</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>CKAM owner</t>
+          <t>DBA; Dev lead</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Weekly</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>GET /api/admin/logs/audit (exists); review record NOT EVIDENCED; LOGS_VIEWED rows record that a review screen was opened</t>
+          <t>docs/security/evidence/infra/db_03_append_only_privilege_tests.out.txt; db_04_least_priv_flag_bypass.out.txt; migration a3c5e7f9b1d4; backend/tests/observability/test_vapt_append_only.py (IF-05/IF-06/AU-10 MITIGATED); migration c6e8a0b2d4f6 (DB guard on asset.status / holder / status_since); ops/db/role_split.sql and check_least_privilege.sql; docs/security/evidence/closure/db/WPB_RESULTS.md</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>N/A (configuration)</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>No review performed or recorded</t>
+          <t>Production owner role can still drop triggers until the role split (EXT-07, EXT-45); the lifecycle guard is marker-based (R-36); nothing deployed</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>EXT-22</t>
+          <t>EXT-07 role split; EXT-01</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CC7-04</t>
+          <t>CC7-03</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2873,32 +3054,32 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Problems are detected quickly</t>
+          <t>Audit logs are reviewed</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Alerts for 5xx spikes, lockouts, backup failure, ERP sync failure, service down</t>
+          <t>Weekly review of SECURITY rows (failed logins, lockouts, access changes, permission denied)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>IT/Infra</t>
+          <t>CKAM owner</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Weekly</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>CKAM; servers</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED (data exists in error_log, system_event)</t>
+          <t>GET /api/admin/logs/audit (exists); review record NOT EVIDENCED; LOGS_VIEWED rows record that a review screen was opened; docs/security/policies/05_Incident_Response_Plan.md (DRAFT) names the weekly review; not operating</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2913,7 +3094,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>No alerting</t>
+          <t>No review performed or recorded</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -2922,6 +3103,11 @@
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -2930,7 +3116,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>CC7-05</t>
+          <t>CC7-04</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2940,37 +3126,37 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Vulnerabilities are found and fixed</t>
+          <t>Problems are detected quickly</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Monthly dependency audit (npm audit, pip-audit); fix SLAs by severity</t>
+          <t>Alerts for 5xx spikes, lockouts, backup failure, ERP sync failure, service down</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>IT/Infra</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>CKAM; servers</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/infra/dependency_audit.md (one-off 2026-10-15)</t>
+          <t>NOT EVIDENCED (data exists in error_log, system_event)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2980,24 +3166,29 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Not scheduled; no SLA</t>
+          <t>No alerting: audit-write failure lines (log_write_failed), REFRESH_REUSE and RATE_LIMITED rows are not alerted on (EXT-22, EXT-48)</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>EXT-09, EXT-12</t>
+          <t>EXT-22</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>CC7-06</t>
+          <t>CC7-05</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3007,22 +3198,22 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Independent penetration testing</t>
+          <t>Vulnerabilities are found and fixed</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>External VAPT by an independent firm</t>
+          <t>Monthly dependency audit (npm audit, pip-audit); fix SLAs by severity</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -3032,12 +3223,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Internal VAPT only (docs/security/evidence/)</t>
+          <t>docs/security/evidence/infra/dependency_audit.md (one-off 2026-10-15); docs/security/evidence/closure/backend/dependency_recheck.md; docs/security/evidence/closure/infra/npm_audit_recheck.md; docs/security/policies/06_Vulnerability_Management_Procedure.md (DRAFT)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3047,24 +3238,29 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>No independent test</t>
+          <t>Not scheduled; no SLA</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>EXT-14</t>
+          <t>EXT-09, EXT-12</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CC7-07</t>
+          <t>CC7-06</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3074,32 +3270,32 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Systems are patched</t>
+          <t>Independent penetration testing</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>OS, Python runtime, PostgreSQL and NAS firmware patched to policy</t>
+          <t>External VAPT by an independent firm</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>IT/Infra</t>
+          <t>Management</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>10.0.1.98, 10.0.0.205, NAS</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>Internal VAPT only (docs/security/evidence/); Internal VAPT plus two internal closure retests (docs/security/evidence/closure/retest1, retest2); no independent firm</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -3114,15 +3310,20 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Not evidenced</t>
+          <t>No independent test</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>EXT-09</t>
+          <t>EXT-14</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -3131,7 +3332,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>CC7-08</t>
+          <t>CC7-07</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3141,32 +3342,32 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Incidents are handled</t>
+          <t>Systems are patched</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Incident response plan, severity, containment, CERT-In reporting, post-incident review</t>
+          <t>OS, Python runtime, PostgreSQL and NAS firmware patched to policy</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>ISMS lead</t>
+          <t>IT/Infra</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Per incident; annual test</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Organisation</t>
+          <t>10.0.1.98, 10.0.0.205, NAS</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED; IF-01 not yet handled as an incident</t>
+          <t>NOT EVIDENCED</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -3181,15 +3382,20 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>No plan</t>
+          <t>Not evidenced</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>EXT-20, EXT-03</t>
+          <t>EXT-09</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -3198,7 +3404,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>CC7-09</t>
+          <t>CC7-08</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -3208,32 +3414,32 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Malware is prevented</t>
+          <t>Incidents are handled</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Antimalware/EDR on servers and NAS</t>
+          <t>Incident response plan, severity, containment, CERT-In reporting, post-incident review</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>IT/Infra</t>
+          <t>ISMS lead</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Per incident; annual test</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Servers</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>NOT EVIDENCED; IF-01 not yet handled as an incident; docs/security/policies/05_Incident_Response_Plan.md and templates/incident_record.md (DRAFT); CKAM_URGENT_PRODUCTION_SECURITY_RUNBOOK.md phase 13 (prepared, not executed)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -3248,15 +3454,20 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Not evidenced</t>
+          <t>No plan</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>EXT-37</t>
+          <t>EXT-20, EXT-03</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -3265,47 +3476,47 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>CC8-01</t>
+          <t>CC7-09</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Security (CC8 Change management)</t>
+          <t>Security (CC7 System operations)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Changes are authorised</t>
+          <t>Malware is prevented</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Owner approves each push; separate owner approval for each production deploy</t>
+          <t>Antimalware/EDR on servers and NAS</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>CKAM owner</t>
+          <t>IT/Infra</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Per change</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>Servers</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE.md; git history; approval itself recorded only in chat sessions</t>
+          <t>NOT EVIDENCED</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3315,49 +3526,54 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Approval not recorded as evidence</t>
+          <t>Not evidenced</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Change record (EXT-35)</t>
+          <t>EXT-37</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CC8-02</t>
+          <t>CC7-10</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Security (CC8 Change management)</t>
+          <t>Security (CC7 System operations)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Changes are tested before release</t>
+          <t>Failures of the audit trail itself are visible</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Backend pytest on ckam_test; frontend tsc + vitest; E2E; security regression tests</t>
+          <t>If an audit or log row cannot be written, the failure is reported on its first occurrence and then at most once a minute with a running count (error log kind log_write_failed plus a system_event row)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>Dev lead; IT/Infra</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Per change</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -3367,39 +3583,44 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE.md rule 4; backend/tests (about 1,783 tests; final run number from the lead); frontend 1,239 tests in 90 files; frontend/e2e incl. security.spec.ts (14/14 security journeys + 11 permanent journeys, 1 skipped); docs/security/CKAM_VAPT_REPORT.md</t>
+          <t>backend/app/observability/writer.py; backend/tests/observability/test_log_write_failure_reporting.py (ca94574)</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>YES (code) / NO (production)</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>NO (no CI run history)</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>No CI; test results kept only in reports, not per change (IF-17)</t>
+          <t>Not deployed; no alert on the line (EXT-48); the Logs &gt; Diagnostics screen does not show the count yet</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>CI (EXT-28); attach test output to change record</t>
+          <t>EXT-01, EXT-48</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>NEW 2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CC8-03</t>
+          <t>CC8-01</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -3409,17 +3630,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Database changes are controlled</t>
+          <t>Changes are authorised</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Schema change only by Alembic migration; never create_all at runtime</t>
+          <t>Owner approves each push; separate owner approval for each production deploy</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>CKAM owner</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -3429,44 +3650,49 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE.md rule 3; backend/app/alembic/versions (41 committed migrations at HEAD d04779a, single head); alembic current at deploy</t>
+          <t>CLAUDE.md; git history; approval itself recorded only in chat sessions; docs/security/policies/04_Change_Management_Procedure.md and templates/change_record.md (DRAFT); 22 local security commits awaiting push approval</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - alembic_version + git history</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Approval not recorded as evidence</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Change record (EXT-35)</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>CC8-04</t>
+          <t>CC8-02</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3476,32 +3702,32 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Deployments are reproducible and reversible</t>
+          <t>Changes are tested before release</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Backup, exact release by commit, migration, restart, smoke checks, rollback folders</t>
+          <t>Backend pytest on ckam_test; frontend tsc + vitest; E2E; security regression tests</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>IT/Infra; Dev lead</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Per deploy</t>
+          <t>Per change</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>10.0.1.98</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (deploy steps and 2026-10-14 notes); system_event app_started with version</t>
+          <t>CLAUDE.md rule 4; backend/tests (about 1,783 tests; final run number from the lead); frontend 1,239 tests in 90 files; frontend/e2e incl. security.spec.ts (14/14 security journeys + 11 permanent journeys, 1 skipped); docs/security/CKAM_VAPT_REPORT.md; Final local run at HEAD fd34520: backend 2541 passed, 1 skipped; frontend tsc clean, vitest 1257 passed in 92 files, npm run build and check:build OK; Playwright 11 passed, 1 skipped; security journeys 14/14 (supersedes the 2026-10-15 figures)</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -3511,20 +3737,25 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL (system_event app_started; launcher log)</t>
+          <t>NO (no CI run history)</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Release script and launcher not in git (IF-15); runbook out of date</t>
+          <t>No CI; test results kept only in reports, not per change (IF-17)</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>EXT-13, EXT-35</t>
+          <t>CI (EXT-28); attach test output to change record</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -3533,7 +3764,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>CC8-05</t>
+          <t>CC8-03</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3543,64 +3774,69 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Emergency changes are controlled</t>
+          <t>Database changes are controlled</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Emergency change procedure (e.g. IF-01) with after-the-fact approval and review</t>
+          <t>Schema change only by Alembic migration; never create_all at runtime</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>CKAM owner</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Per emergency</t>
+          <t>Per change</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>CLAUDE.md rule 3; backend/app/alembic/versions (41 committed migrations at HEAD d04779a, single head); alembic current at deploy; 43 committed migrations at HEAD fd34520, single head c6e8a0b2d4f6 (4 added by the security programme, not deployed)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SOURCE EXISTS - alembic_version + git history</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>No procedure</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>EXT-35</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>CC8-06</t>
+          <t>CC8-04</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3610,32 +3846,32 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Code is developed securely</t>
+          <t>Deployments are reproducible and reversible</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Security baseline, guardrails, file-security review, authorization tests</t>
+          <t>Backup, exact release by commit, migration, restart, smoke checks, rollback folders</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>IT/Infra; Dev lead</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Per change</t>
+          <t>Per deploy</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>10.0.1.98</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>docs/security/CKAM_SECURITY_BASELINE.md; docs/ai/DEVELOPMENT_GUARDRAILS.md (security rules committed in da790d1)</t>
+          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (deploy steps and 2026-10-14 notes); system_event app_started with version; ops/windows/ reference launcher, deploy, verify and rollback templates (secret-free; parser and -WhatIf validated); docs/security/CKAM_URGENT_PRODUCTION_SECURITY_RUNBOOK.md (prepared, NOT executed)</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -3645,20 +3881,25 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PARTIAL (system_event app_started; launcher log)</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Baseline not yet approved; not evidenced per change</t>
+          <t>Live launcher and release script not in git (EXT-13); reference templates not yet confirmed against the server; runbook never executed</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Approve baseline; checklist in change record</t>
+          <t>EXT-13, EXT-35</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -3667,7 +3908,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>CC8-07</t>
+          <t>CC8-05</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -3677,22 +3918,22 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Dependencies are controlled</t>
+          <t>Emergency changes are controlled</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Lock/constraints for Python; npm lock; audit before adding/upgrading</t>
+          <t>Emergency change procedure (e.g. IF-01) with after-the-fact approval and review</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>CKAM owner</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Per change</t>
+          <t>Per emergency</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -3702,12 +3943,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>frontend/package-lock.json; backend/constraints.txt (IF-11 FIXED in code)</t>
+          <t>NOT EVIDENCED; docs/security/policies/04_Change_Management_Procedure.md emergency path (DRAFT); EXT-42 (IF-01 emergency change record) prepared</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3717,64 +3958,69 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Production install not yet using constraints.txt</t>
+          <t>No procedure</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>EXT-12</t>
+          <t>EXT-35</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>CC9-01</t>
+          <t>CC8-06</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Security (CC9 Risk mitigation)</t>
+          <t>Security (CC8 Change management)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Suppliers are managed</t>
+          <t>Code is developed securely</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Supplier register and review (ERP team, NAS, GitHub, AI coding assistant provider, Google Fonts)</t>
+          <t>Security baseline, guardrails, file-security review, authorization tests</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Per change</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Organisation</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>docs/security/CKAM_SECURITY_BASELINE.md; docs/ai/DEVELOPMENT_GUARDRAILS.md (security rules committed in da790d1); docs/security/CKAM_SECURITY_BASELINE.md updated 2026-10-16 with the closure rules</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3784,64 +4030,69 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>No supplier review</t>
+          <t>Baseline not yet approved; not evidenced per change</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>EXT-34</t>
+          <t>Approve baseline; checklist in change record</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>CC9-02</t>
+          <t>CC8-07</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Security (CC9 Risk mitigation)</t>
+          <t>Security (CC8 Change management)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Business disruption is planned for</t>
+          <t>Dependencies are controlled</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>BCP covering CKAM outage, data loss and ransomware</t>
+          <t>Lock/constraints for Python; npm lock; audit before adding/upgrading</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Management; IT/Infra</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Per change</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Organisation</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>frontend/package-lock.json; backend/constraints.txt (IF-11 FIXED in code); docs/security/evidence/closure/backend/dependency_recheck.md (python-jose / ecdsa no fixed version, not reachable, ACCEPTED; PyJWT replacement recommended, EXT-47)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -3851,158 +4102,173 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>No BCP</t>
+          <t>Production install not yet using constraints.txt</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>EXT-29</t>
+          <t>EXT-12</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>A1-01</t>
+          <t>CC9-01</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Security (CC9 Risk mitigation)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Capacity is sufficient</t>
+          <t>Suppliers are managed</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Monitor disk, DB size, slow requests and slow SQL</t>
+          <t>Supplier register and review (ERP team, NAS, GitHub, AI coding assistant provider, Google Fonts)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>IT/Infra</t>
+          <t>Management</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>CKAM; servers</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>error_log slow_request / slow_sql rows; GET /api/admin/diagnostics/db</t>
+          <t>NOT EVIDENCED; docs/security/policies/09_Supplier_Security_Review.md (DRAFT)</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - error_log kept 180 days</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>No thresholds or review</t>
+          <t>No supplier review</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>EXT-22</t>
+          <t>EXT-34</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>A1-02</t>
+          <t>CC9-02</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Security (CC9 Risk mitigation)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Data is backed up daily</t>
+          <t>Business disruption is planned for</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Nightly pg dump of ckassetmanagement, 30 days kept</t>
+          <t>BCP covering CKAM outage, data loss and ransomware</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>IT/Infra</t>
+          <t>Management; IT/Infra</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>10.0.0.205</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (backup.log on DB server)</t>
+          <t>NOT EVIDENCED; docs/security/policies/08_Business_Continuity_and_DR_Plan.md (DRAFT)</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - backup.log; no observation period</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Same server, unencrypted; NAS files not evidenced (IF-08)</t>
+          <t>No BCP</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>EXT-08</t>
+          <t>EXT-29</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>A1-03</t>
+          <t>A1-01</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4012,12 +4278,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Backups survive loss of the server</t>
+          <t>Capacity is sufficient</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Encrypted off-server copy of DB dumps and NAS documents</t>
+          <t>Monitor disk, DB size, slow requests and slow SQL</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -4027,49 +4293,54 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Backup target</t>
+          <t>CKAM; servers</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>error_log slow_request / slow_sql rows; GET /api/admin/diagnostics/db</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SOURCE EXISTS - error_log kept 180 days</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>No off-server copy</t>
+          <t>No thresholds or review</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>EXT-08</t>
+          <t>EXT-22</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>A1-04</t>
+          <t>A1-02</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -4079,12 +4350,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Backups can be restored</t>
+          <t>Data is backed up daily</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Quarterly restore test into a throw-away database with row-count checks</t>
+          <t>Nightly pg dump of ckassetmanagement, 30 days kept</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -4094,7 +4365,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -4104,22 +4375,22 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Dev drill only (docs/ai/AM-09_RC_FULL_AUDIT_REPORT.md; ops/test_backup_restore.sh, dev-only)</t>
+          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (backup.log on DB server)</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SOURCE EXISTS - backup.log; no observation period</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Never restored in production</t>
+          <t>Same server, unencrypted; NAS files not evidenced (IF-08)</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
@@ -4129,14 +4400,19 @@
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>A1-05</t>
+          <t>A1-03</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -4146,32 +4422,32 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Recovery objectives are defined</t>
+          <t>Backups survive loss of the server</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>DR plan with RTO/RPO, reboot test, rollback incl. DB restore</t>
+          <t>Encrypted off-server copy of DB dumps and NAS documents</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Management; IT/Infra</t>
+          <t>IT/Infra</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>Backup target</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (rollback needs DB restore; reboot test still open)</t>
+          <t>NOT EVIDENCED; docs/security/CKAM_BACKUP_RESTORE_PLAN.md (prepared, not implemented)</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -4186,15 +4462,20 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>No RTO/RPO; reboot test open</t>
+          <t>No off-server copy</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>EXT-29</t>
+          <t>EXT-08</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
@@ -4203,7 +4484,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>A1-06</t>
+          <t>A1-04</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -4213,12 +4494,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>The service restarts and reports health</t>
+          <t>Backups can be restored</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Scheduled task restart; /api/health; diagnostics/health; startup/shutdown events</t>
+          <t>Quarterly restore test into a throw-away database with row-count checks</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -4228,74 +4509,79 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>10.0.1.98</t>
+          <t>10.0.0.205</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md; system_event startup/shutdown; GET /api/admin/diagnostics/health</t>
+          <t>Dev drill only (docs/ai/AM-09_RC_FULL_AUDIT_REPORT.md; ops/test_backup_restore.sh, dev-only); docs/security/CKAM_BACKUP_RESTORE_PLAN.md and policies/templates/restore_test_record.md (prepared, never run)</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - system_event kept 180 days</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>No external uptime check</t>
+          <t>Never restored in production</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>EXT-22</t>
+          <t>EXT-08</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>C1-01</t>
+          <t>A1-05</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Confidentiality</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Confidential information is identified and restricted</t>
+          <t>Recovery objectives are defined</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Vendor commercial data, PO values, invoices, documents restricted by role, company and work area</t>
+          <t>DR plan with RTO/RPO, reboot test, rollback incl. DB restore</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>ISMS lead; Dev lead</t>
+          <t>Management; IT/Infra</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Annual classification; continuous enforcement</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -4305,74 +4591,79 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/access/tests.csv; AC-1 fix (vendor contacts no longer readable by Own Assets Only, pending retest)</t>
+          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md (rollback needs DB restore; reboot test still open); docs/security/policies/08_Business_Continuity_and_DR_Plan.md (DRAFT)</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - DOCUMENT_DOWNLOADED and EXPORT rows</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>No classification scheme</t>
+          <t>No RTO/RPO; reboot test open</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Classification (A.5.12)</t>
+          <t>EXT-29</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>C1-02</t>
+          <t>A1-06</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Confidentiality</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Confidential information is retained and disposed of per policy</t>
+          <t>The service restarts and reports health</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Log retention 180 days; audit kept forever; guarded audit purge; no business-data deletion</t>
+          <t>Scheduled task restart; /api/health; diagnostics/health; startup/shutdown events</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Management; Legal</t>
+          <t>IT/Infra</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>10.0.1.98</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md section 4; system_event retention/purge_finished</t>
+          <t>docs/ai/PRODUCTION_INFRASTRUCTURE.md; system_event startup/shutdown; GET /api/admin/diagnostics/health</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -4382,20 +4673,25 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - purge_finished events</t>
+          <t>SOURCE EXISTS - system_event kept 180 days</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>No approved retention schedule</t>
+          <t>No external uptime check</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>EXT-21, EXT-31</t>
+          <t>EXT-22</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -4404,7 +4700,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>C1-03</t>
+          <t>C1-01</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -4414,22 +4710,22 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Exports are controlled and traceable</t>
+          <t>Confidential information is identified and restricted</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Role-restricted exports; every export audited with filters and row count; formula injection neutralised</t>
+          <t>Vendor commercial data, PO values, invoices, documents restricted by role, company and work area</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>ISMS lead; Dev lead</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Annual classification; continuous enforcement</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -4439,39 +4735,44 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md (EXPORT rows); docs/security/evidence/input/formula_export_cell.txt</t>
+          <t>docs/security/evidence/access/tests.csv; AC-1 fix (vendor contacts no longer readable by Own Assets Only, pending retest); AC-1 fix retested in closure retests 1 and 2 (not deployed)</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - no observation period</t>
+          <t>SOURCE EXISTS - DOCUMENT_DOWNLOADED and EXPORT rows</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No classification scheme</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Classification (A.5.12)</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>C1-04</t>
+          <t>C1-02</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -4481,22 +4782,22 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Secrets never reach code, logs or audit</t>
+          <t>Confidential information is retained and disposed of per policy</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>No secrets in repo; redaction by key and value pattern; diagnostics bundle clean</t>
+          <t>Log retention 180 days; audit kept forever; guarded audit purge; no business-data deletion</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>Management; Legal</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -4506,39 +4807,44 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Secrets scan (none in working tree or 282 commits); docs/security/evidence/auth/tests.csv AU-T049, AU-T089, AU-T090; backend/tests/observability/test_redaction.py</t>
+          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md section 4; system_event retention/purge_finished</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - test runs</t>
+          <t>SOURCE EXISTS - purge_finished events</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No approved retention schedule</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Keep scan in release checklist</t>
+          <t>EXT-21, EXT-31</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>C1-05</t>
+          <t>C1-03</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -4548,79 +4854,84 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Development copies of data are protected</t>
+          <t>Exports are controlled and traceable</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Dev PC ACL, disk encryption, minimum real data in dev</t>
+          <t>Role-restricted exports; every export audited with filters and row count; formula injection neutralised</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Dev lead; IT</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Dev PC 10.0.0.47</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>IF-09; docs/ai/ERP_INTEGRATION.md (dev ERP copy of real data)</t>
+          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md (EXPORT rows); docs/security/evidence/input/formula_export_cell.txt</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SOURCE EXISTS - no observation period</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Dev .env and dumps readable by too many accounts</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>EXT-10</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>PI1-01</t>
+          <t>C1-04</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Processing Integrity</t>
+          <t>Confidentiality</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Inputs are complete and valid</t>
+          <t>Secrets never reach code, logs or audit</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Schema validation (pydantic), 422 with every problem, size limits, quantity 1..1,000</t>
+          <t>No secrets in repo; redaction by key and value pattern; diagnostics bundle clean</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -4635,12 +4946,12 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>CKAM API</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/input/tests.csv; docs/security/evidence/auth/tests.csv AU-T069..AU-T078</t>
+          <t>Secrets scan (none in working tree or 282 commits); docs/security/evidence/auth/tests.csv AU-T049, AU-T089, AU-T090; backend/tests/observability/test_redaction.py; Closure secret scan (regex only): working tree, 299+ commits, built frontend, image layers and container env hold no real secret (docs/security/evidence/closure/retest2/infra/raw/secret_scan_summary.txt); refresh-token ids stored only as SHA-256</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -4650,7 +4961,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>N/A (configuration)</t>
+          <t>SOURCE EXISTS - test runs</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4660,10 +4971,15 @@
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Keep scan in release checklist</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4672,74 +4988,79 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>PI1-02</t>
+          <t>C1-05</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Processing Integrity</t>
+          <t>Confidentiality</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>A request is processed once</t>
+          <t>Development copies of data are protected</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Idempotency keys per actor on write requests; replay and conflict audited</t>
+          <t>Dev PC ACL, disk encryption, minimum real data in dev</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>Dev lead; IT</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>CKAM API</t>
+          <t>Dev PC 10.0.0.47</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>backend/app/core/idempotency.py; docs/security/evidence/access/tests.csv (7 idempotency/business-logic cases); audit IDEMPOTENT_REPLAY / IDEMPOTENT_CONFLICT</t>
+          <t>IF-09; docs/ai/ERP_INTEGRATION.md (dev ERP copy of real data); docs/security/evidence/closure/infra/IF-09_ACL_PLAN.md (plan only; nothing changed on the dev PC)</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - ACCESS rows</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Dev .env and dumps readable by too many accounts</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>EXT-10</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>PI1-03</t>
+          <t>PI1-01</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -4749,17 +5070,17 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Asset history is complete and unalterable</t>
+          <t>Inputs are complete and valid</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>apply_event / apply_events single writer of status, holder, status_since; asset_event append-only; asset_code immutable</t>
+          <t>Schema validation (pydantic), 422 with every problem, size limits, quantity 1..1,000</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Dev lead; DBA</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -4769,12 +5090,12 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>CKAM; PostgreSQL</t>
+          <t>CKAM API</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>backend/app/lifecycle/service.py; docs/security/evidence/infra/db_02_triggers_constraints.out.txt; db_03 A9 (status column has no DB-level guard)</t>
+          <t>docs/security/evidence/input/tests.csv; docs/security/evidence/auth/tests.csv AU-T069..AU-T078</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -4784,20 +5105,25 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - asset_event</t>
+          <t>N/A (configuration)</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Status column writable directly by DB owner (A9)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Role split (EXT-07)</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4806,7 +5132,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>PI1-04</t>
+          <t>PI1-02</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4816,12 +5142,12 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Bulk operations are all-or-nothing</t>
+          <t>A request is processed once</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Receive and Add Assets check everything first then write in one transaction</t>
+          <t>Idempotency keys per actor on write requests; replay and conflict audited</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -4836,12 +5162,12 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>CKAM API</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/DECISIONS.md 2026-10-14 (6)</t>
+          <t>backend/app/core/idempotency.py; docs/security/evidence/access/tests.csv (7 idempotency/business-logic cases); audit IDEMPOTENT_REPLAY / IDEMPOTENT_CONFLICT</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -4851,7 +5177,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - audit RECEIVE / BATCH_ADD rows</t>
+          <t>SOURCE EXISTS - ACCESS rows</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -4865,6 +5191,11 @@
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4873,7 +5204,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>PI1-05</t>
+          <t>PI1-03</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4883,17 +5214,17 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Unique identity of assets</t>
+          <t>Asset history is complete and unalterable</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Unique asset code, case-insensitive unique serial (N/A exempt), unique PO per company</t>
+          <t>apply_event / apply_events single writer of status, holder, status_since; asset_event append-only; asset_code immutable</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>Dev lead; DBA</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -4903,12 +5234,12 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>CKAM; PostgreSQL</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/infra/db_02_triggers_constraints.out.txt; docs/security/evidence/infra/db_05_data_integrity.out.txt</t>
+          <t>backend/app/lifecycle/service.py; docs/security/evidence/infra/db_02_triggers_constraints.out.txt; db_03 A9 (status column has no DB-level guard); migration c6e8a0b2d4f6_asset_lifecycle_fields_guard.py; backend/tests/lifecycle/test_obs_status_guard.py (closure, not deployed)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4918,20 +5249,25 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS</t>
+          <t>SOURCE EXISTS - asset_event</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>db_05 shows 2 dev-stack observations to explain (two primary owners; user id 1 without a CREATE audit row)</t>
+          <t>DB guard not deployed; anyone with SQL as the app role can set the marker (R-36); the strong barrier is the role split (EXT-07)</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Explain/clean dev observations</t>
+          <t>Role split (EXT-07)</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4940,7 +5276,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>PI1-06</t>
+          <t>PI1-04</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -4950,17 +5286,17 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>ERP data is read, never written</t>
+          <t>Bulk operations are all-or-nothing</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>ERP role read-only; every connection sets default_transaction_read_only; code issues SELECT only; create re-reads the copy</t>
+          <t>Receive and Add Assets check everything first then write in one transaction</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Dev lead; ERP owner</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -4970,44 +5306,49 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>ERP 10.0.1.69</t>
+          <t>CKAM</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/ERP_INTEGRATION.md; backend/app/erp/source.py; backend/tests/erp/test_vapt_erp_limits.py (IF-10 FIXED: timeouts, read-only); system_event erp_sync</t>
+          <t>docs/ai/DECISIONS.md 2026-10-14 (6)</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - erp_sync_run, system_event</t>
+          <t>SOURCE EXISTS - audit RECEIVE / BATCH_ADD rows</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>No TLS option (IF-16, OPEN EXTERNAL); SELECT-only grant on ERP side not evidenced; timeouts not deployed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>EXT-25</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>PI1-08</t>
+          <t>PI1-05</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -5017,12 +5358,12 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Concurrent requests do not create duplicates</t>
+          <t>Unique identity of assets</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Creating a vendor or brand with the same name at the same moment is serialized; only one is created</t>
+          <t>Unique asset code, case-insensitive unique serial (N/A exempt), unique PO per company</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -5037,44 +5378,49 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>CKAM API</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/core/test_security_concurrency.py (RACE-1 FIXED, commit da790d1)</t>
+          <t>docs/security/evidence/infra/db_02_triggers_constraints.out.txt; docs/security/evidence/infra/db_05_data_integrity.out.txt; backend/tests/masters/test_wpf2_category_names.py (one active category/sub-category name per work area); backend/tests/core/test_wpf2_serial_race_message.py (friendly 422 for the loser of a same-serial race)</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>YES (code) / NO (production)</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>N/A (configuration)</t>
+          <t>SOURCE EXISTS</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>Not deployed</t>
+          <t>db_05 shows 2 dev-stack observations to explain (two primary owners; user id 1 without a CREATE audit row)</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>EXT-01</t>
+          <t>Explain/clean dev observations</t>
         </is>
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>PI1-07</t>
+          <t>PI1-06</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5084,17 +5430,17 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Exports are safe to open</t>
+          <t>ERP data is read, never written</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Leading apostrophe on values starting with = + - @ in every export</t>
+          <t>ERP role read-only; every connection sets default_transaction_read_only; code issues SELECT only; create re-reads the copy</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Dev lead</t>
+          <t>Dev lead; ERP owner</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -5104,126 +5450,136 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>ERP 10.0.1.69</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>docs/security/evidence/input/formula_export_cell.txt</t>
+          <t>docs/ai/ERP_INTEGRATION.md; backend/app/erp/source.py; backend/tests/erp/test_vapt_erp_limits.py (IF-10 FIXED: timeouts, read-only); system_event erp_sync; backend/tests/erp/test_erp_tls_settings.py (PO_SOURCE_SSLMODE / PO_SOURCE_SSLROOTCERT, default prefer)</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>N/A (configuration)</t>
+          <t>SOURCE EXISTS - erp_sync_run, system_event</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>TLS settable but not mandatory; ERP owner must confirm TLS and the SELECT-only grant (EXT-25); timeouts not deployed</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>EXT-25</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>PI1-08</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Privacy</t>
+          <t>Processing Integrity</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>People are told what personal data is kept</t>
+          <t>Concurrent requests do not create duplicates</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Privacy notice for staff and store users (names, codes, emails, phones, IP addresses in logs)</t>
+          <t>Same-name creation is serialized (vendor, brand, category / sub-category per work area, also in Excel imports); parallel receive, idempotency, serial and move bursts create no duplicates and no over-receiving</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Legal; HR</t>
+          <t>Dev lead</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>CKAM</t>
+          <t>CKAM API</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>NOT EVIDENCED</t>
+          <t>backend/tests/core/test_security_concurrency.py (RACE-1 FIXED, commit da790d1); backend/tests/masters/test_import_duplicate_names.py; backend/tests/masters/test_wpf2_category_names.py; docs/security/evidence/closure/retest2/sessions/concurrency_results.md (bursts x20: no duplicates, no 500, no deadlock)</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES (code) / NO (production)</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>N/A (configuration)</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>No notice</t>
+          <t>Not deployed</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>EXT-31</t>
+          <t>EXT-01</t>
         </is>
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>NOT IN SCOPE</t>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>P-02</t>
+          <t>PI1-07</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Privacy</t>
+          <t>Processing Integrity</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Personal data is limited and access-controlled</t>
+          <t>Exports are safe to open</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Only needed fields; logs head-office admin only; redaction</t>
+          <t>Leading apostrophe on values starting with = + - @ in every export</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -5243,39 +5599,44 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md section 9</t>
+          <t>docs/security/evidence/input/formula_export_cell.txt</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>SOURCE EXISTS - LOGS_VIEWED rows</t>
+          <t>N/A (configuration)</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>No PII review</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>Review fields with legal (EXT-31)</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>P-03</t>
+          <t>P-01</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -5285,22 +5646,22 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Personal data requests and retention are handled</t>
+          <t>People are told what personal data is kept</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Process for access/correction requests and PII retention within append-only design</t>
+          <t>Privacy notice for staff and store users (names, codes, emails, phones, IP addresses in logs)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Legal; HR</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Per request</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -5325,7 +5686,7 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>No process</t>
+          <t>No notice</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
@@ -5334,6 +5695,11 @@
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>NOT IN SCOPE</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
         <is>
           <t>NOT IN SCOPE</t>
         </is>
@@ -5342,72 +5708,221 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Personal data is limited and access-controlled</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Only needed fields; logs head-office admin only; redaction</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Dev lead</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>CKAM</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>docs/ai/LOGGING_AND_DIAGNOSTICS.md section 9</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE EXISTS - LOGS_VIEWED rows</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>No PII review</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Review fields with legal (EXT-31)</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Personal data requests and retention are handled</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Process for access/correction requests and PII retention within append-only design</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Per request</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>CKAM</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>NOT EVIDENCED</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>No process</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>EXT-31</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>NOT IN SCOPE</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>NOT IN SCOPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
           <t>P-04</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Privacy</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Personal data is not disclosed to third parties unnecessarily</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>Fonts loaded from Google send user IP addresses to a third party</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>Dev lead</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr">
         <is>
           <t>CKAM frontend</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>frontend/index.html; frontend/src/fonts.css (self-hosted Inter + IBM Plex Mono, 79dbae7); CSP without Google hosts (b401e9f); docs/security/evidence/closure/retest2/infra/raw/fonts_csp_playwright_summary.txt (0 Google requests)</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>YES (code) / NO (production)</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>Third-party font CDN</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>EXT-11</t>
-        </is>
-      </c>
-      <c r="M74" s="2" t="inlineStr">
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Not deployed: production 3b5e842 still loads Google Fonts</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>EXT-01 (EXT-11 code side done)</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>READY IN CODE - NOT DEPLOYED</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M74"/>
+  <autoFilter ref="A1:N76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>